<commit_message>
Cleanup tests and scripts - Remove redundant test files and unused libraries - Update run scripts to work from tests directory - Fix common.robot reference to deleted TimelineAnalyzer - Update GitHub workflows - Simplify requirements.txt
</commit_message>
<xml_diff>
--- a/timeline.xlsx
+++ b/timeline.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://epam-my.sharepoint.com/personal/alexey_mogilny_epam_com/Documents/Projects/_EPM-AI_/Timeline generator/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\powerpoint-timeline-generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="252" documentId="8_{69AF3E5A-AD33-435A-ABA5-5668914A2249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE001E43-D24F-4863-BCB6-FE106318B532}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F2F9DA0-C833-49AF-B741-9C293D00D424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14505" yWindow="-2280" windowWidth="14610" windowHeight="15585" xr2:uid="{4579CA89-1D2B-494E-904A-50BDFCDF60D4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4579CA89-1D2B-494E-904A-50BDFCDF60D4}"/>
   </bookViews>
   <sheets>
     <sheet name="TimelineData" sheetId="1" r:id="rId1"/>
@@ -210,10 +210,6 @@
   </cellStyles>
   <dxfs count="7">
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -222,6 +218,17 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -243,13 +250,6 @@
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -264,15 +264,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{87A4A6B7-9301-4921-B86F-DDACC1ACB6F2}" name="Table1" displayName="Table1" ref="A1:F22" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{87A4A6B7-9301-4921-B86F-DDACC1ACB6F2}" name="Table1" displayName="Table1" ref="A1:F22" totalsRowShown="0" headerRowDxfId="6">
   <autoFilter ref="A1:F22" xr:uid="{87A4A6B7-9301-4921-B86F-DDACC1ACB6F2}"/>
   <tableColumns count="6">
-    <tableColumn id="6" xr3:uid="{B91E3DCD-028E-4B61-BF11-A448EFDDBADE}" name="Task Name" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{F71040F1-BFC9-44BF-8C11-74A45B4197BC}" name="Start Date" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{B91E3DCD-028E-4B61-BF11-A448EFDDBADE}" name="Task Name" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{F71040F1-BFC9-44BF-8C11-74A45B4197BC}" name="Start Date" dataDxfId="4"/>
     <tableColumn id="4" xr3:uid="{31F432EB-47CD-4910-9217-CEDF208EAA5D}" name="End Date" dataDxfId="3"/>
     <tableColumn id="5" xr3:uid="{850626D4-1BC9-453F-A63E-CECA0C728AB2}" name="Type" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{E67EE7CB-AF3B-48DA-BC65-2F2E20DBA1CE}" name="Color" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{F19A7BAE-2A9E-4FF6-9DA6-A7C7893C00E5}" name="Swimlane" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{E67EE7CB-AF3B-48DA-BC65-2F2E20DBA1CE}" name="Color" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{F19A7BAE-2A9E-4FF6-9DA6-A7C7893C00E5}" name="Swimlane" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -632,10 +632,10 @@
         <v>15</v>
       </c>
       <c r="B2" s="3">
-        <v>45708</v>
+        <v>45889</v>
       </c>
       <c r="C2" s="3">
-        <v>45719</v>
+        <v>45903</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>27</v>
@@ -650,10 +650,10 @@
         <v>4</v>
       </c>
       <c r="B3" s="3">
-        <v>45708</v>
+        <v>45889</v>
       </c>
       <c r="C3" s="3">
-        <v>45719</v>
+        <v>45903</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>32</v>
@@ -670,10 +670,10 @@
         <v>5</v>
       </c>
       <c r="B4" s="3">
-        <v>45710</v>
+        <v>45891</v>
       </c>
       <c r="C4" s="3">
-        <v>45719</v>
+        <v>45903</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>32</v>
@@ -690,10 +690,10 @@
         <v>6</v>
       </c>
       <c r="B5" s="3">
-        <v>45715</v>
+        <v>45896</v>
       </c>
       <c r="C5" s="3">
-        <v>45719</v>
+        <v>45903</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>32</v>
@@ -710,10 +710,10 @@
         <v>7</v>
       </c>
       <c r="B6" s="3">
-        <v>45715</v>
+        <v>45896</v>
       </c>
       <c r="C6" s="3">
-        <v>45719</v>
+        <v>45903</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>32</v>
@@ -730,10 +730,10 @@
         <v>16</v>
       </c>
       <c r="B7" s="3">
-        <v>45722</v>
+        <v>45906</v>
       </c>
       <c r="C7" s="3">
-        <v>45782</v>
+        <v>45966</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>27</v>
@@ -748,7 +748,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="3">
-        <v>45722</v>
+        <v>45906</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3" t="s">
@@ -766,10 +766,10 @@
         <v>9</v>
       </c>
       <c r="B9" s="3">
-        <v>45722</v>
+        <v>45906</v>
       </c>
       <c r="C9" s="3">
-        <v>45726</v>
+        <v>45910</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>32</v>
@@ -786,10 +786,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="3">
-        <v>45722</v>
+        <v>45906</v>
       </c>
       <c r="C10" s="3">
-        <v>45726</v>
+        <v>45910</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>32</v>
@@ -806,10 +806,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="3">
-        <v>45729</v>
+        <v>45913</v>
       </c>
       <c r="C11" s="3">
-        <v>45782</v>
+        <v>45966</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>32</v>
@@ -826,10 +826,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="3">
-        <v>45729</v>
+        <v>45913</v>
       </c>
       <c r="C12" s="3">
-        <v>45782</v>
+        <v>45966</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>32</v>
@@ -846,10 +846,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="3">
-        <v>45729</v>
+        <v>45913</v>
       </c>
       <c r="C13" s="3">
-        <v>45782</v>
+        <v>45966</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>32</v>
@@ -866,10 +866,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="3">
-        <v>45757</v>
+        <v>45940</v>
       </c>
       <c r="C14" s="3">
-        <v>45782</v>
+        <v>45966</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>32</v>
@@ -886,10 +886,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="3">
-        <v>45771</v>
+        <v>45954</v>
       </c>
       <c r="C15" s="3">
-        <v>45782</v>
+        <v>45966</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>32</v>
@@ -906,10 +906,10 @@
         <v>17</v>
       </c>
       <c r="B16" s="3">
-        <v>45785</v>
+        <v>45969</v>
       </c>
       <c r="C16" s="3">
-        <v>45803</v>
+        <v>45987</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>27</v>
@@ -924,10 +924,10 @@
         <v>18</v>
       </c>
       <c r="B17" s="3">
-        <v>45785</v>
+        <v>45969</v>
       </c>
       <c r="C17" s="3">
-        <v>45796</v>
+        <v>45980</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>32</v>
@@ -944,10 +944,10 @@
         <v>19</v>
       </c>
       <c r="B18" s="3">
-        <v>45785</v>
+        <v>45969</v>
       </c>
       <c r="C18" s="3">
-        <v>45796</v>
+        <v>45980</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>32</v>
@@ -964,7 +964,7 @@
         <v>20</v>
       </c>
       <c r="B19" s="3">
-        <v>45799</v>
+        <v>45983</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3" t="s">
@@ -982,10 +982,10 @@
         <v>21</v>
       </c>
       <c r="B20" s="3">
-        <v>45751</v>
+        <v>45934</v>
       </c>
       <c r="C20" s="3">
-        <v>45782</v>
+        <v>45966</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>32</v>
@@ -1002,10 +1002,10 @@
         <v>22</v>
       </c>
       <c r="B21" s="3">
-        <v>45785</v>
+        <v>45969</v>
       </c>
       <c r="C21" s="3">
-        <v>45796</v>
+        <v>45980</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>32</v>
@@ -1022,10 +1022,10 @@
         <v>23</v>
       </c>
       <c r="B22" s="3">
-        <v>45813</v>
+        <v>45996</v>
       </c>
       <c r="C22" s="3">
-        <v>45859</v>
+        <v>46043</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>32</v>

</xml_diff>